<commit_message>
added removal of pallets with 400 and 360 of quantity, and counter
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
   <si>
     <t>LS1</t>
   </si>
@@ -19,31 +19,142 @@
     <t>Ordem</t>
   </si>
   <si>
+    <t>6878696889</t>
+  </si>
+  <si>
+    <t>Destino</t>
+  </si>
+  <si>
+    <t>Cachoeirinha</t>
+  </si>
+  <si>
+    <t>Caixa</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>Posição</t>
+  </si>
+  <si>
+    <t>Qtd - MIL</t>
+  </si>
+  <si>
+    <t>Case ID</t>
+  </si>
+  <si>
+    <t>Código de Barras</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Destino</t>
-  </si>
-  <si>
-    <t>Itajaí</t>
-  </si>
-  <si>
-    <t>Caixa</t>
-  </si>
-  <si>
-    <t>SKU</t>
-  </si>
-  <si>
-    <t>Posição</t>
-  </si>
-  <si>
-    <t>Qtd - MIL</t>
-  </si>
-  <si>
-    <t>Case ID</t>
-  </si>
-  <si>
-    <t>Código de Barras</t>
+    <t>BLD008</t>
+  </si>
+  <si>
+    <t>0000138827</t>
+  </si>
+  <si>
+    <t>BOX</t>
+  </si>
+  <si>
+    <t>BLF080</t>
+  </si>
+  <si>
+    <t>0000138798</t>
+  </si>
+  <si>
+    <t>BLE055</t>
+  </si>
+  <si>
+    <t>0000138809</t>
+  </si>
+  <si>
+    <t>BLF046</t>
+  </si>
+  <si>
+    <t>0000138813</t>
+  </si>
+  <si>
+    <t>BLD087</t>
+  </si>
+  <si>
+    <t>0000138814</t>
+  </si>
+  <si>
+    <t>FR.01.05.01.03</t>
+  </si>
+  <si>
+    <t>0000138316</t>
+  </si>
+  <si>
+    <t>0000138755</t>
+  </si>
+  <si>
+    <t>FUMO</t>
+  </si>
+  <si>
+    <t>BLD062</t>
+  </si>
+  <si>
+    <t>0000138812</t>
+  </si>
+  <si>
+    <t>NINE</t>
+  </si>
+  <si>
+    <t>BLG072</t>
+  </si>
+  <si>
+    <t>0000138836</t>
+  </si>
+  <si>
+    <t>BLD058</t>
+  </si>
+  <si>
+    <t>0000138837</t>
+  </si>
+  <si>
+    <t>SLIVE</t>
+  </si>
+  <si>
+    <t>BLD001</t>
+  </si>
+  <si>
+    <t>0000138810</t>
+  </si>
+  <si>
+    <t>BLD073</t>
+  </si>
+  <si>
+    <t>0000138811</t>
+  </si>
+  <si>
+    <t>BLF078</t>
+  </si>
+  <si>
+    <t>0000138825</t>
+  </si>
+  <si>
+    <t>BLD007</t>
+  </si>
+  <si>
+    <t>0000138826</t>
+  </si>
+  <si>
+    <t>SLIVE P</t>
+  </si>
+  <si>
+    <t>BLH079</t>
+  </si>
+  <si>
+    <t>0000138807</t>
+  </si>
+  <si>
+    <t>BLE030</t>
+  </si>
+  <si>
+    <t>0000138808</t>
   </si>
 </sst>
 </file>
@@ -124,6 +235,635 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>88000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,7 +1188,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -495,8 +1235,329 @@
         <v>10</v>
       </c>
     </row>
+    <row r="4" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3">
+        <v>10231474</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3">
+        <v>10215641</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3">
+        <v>200</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="3">
+        <v>10224293</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="3">
+        <v>10226339</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3">
+        <v>120</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3">
+        <v>10226359</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3">
+        <v>120</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3">
+        <v>10226363</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="3">
+        <v>10</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>10226363</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="3">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="3">
+        <v>10230675</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="3">
+        <v>10226368</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3">
+        <v>40</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="3">
+        <v>10238738</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="3">
+        <v>40</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="3">
+        <v>10198819</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="3">
+        <v>70</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="3">
+        <v>10198819</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="3">
+        <v>10</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="3">
+        <v>200</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="3">
+        <v>10231475</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="3">
+        <v>20</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="3">
+        <v>10223108</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="3">
+        <v>20</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="3">
+        <v>10226385</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="3">
+        <v>10</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
moved excel file processing logic into main.ts
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="118">
   <si>
     <t>LS1</t>
   </si>
@@ -19,13 +19,13 @@
     <t>Ordem</t>
   </si>
   <si>
-    <t>6878696889</t>
+    <t>6878704262</t>
   </si>
   <si>
     <t>Destino</t>
   </si>
   <si>
-    <t>Cachoeirinha</t>
+    <t>Itajaí</t>
   </si>
   <si>
     <t>Caixa</t>
@@ -46,58 +46,163 @@
     <t>Código de Barras</t>
   </si>
   <si>
+    <t>BOX</t>
+  </si>
+  <si>
+    <t>BLD075</t>
+  </si>
+  <si>
+    <t>0000138907</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>BLD008</t>
-  </si>
-  <si>
-    <t>0000138827</t>
-  </si>
-  <si>
-    <t>BOX</t>
+    <t>BLE050</t>
+  </si>
+  <si>
+    <t>0000138309</t>
   </si>
   <si>
     <t>BLF080</t>
   </si>
   <si>
-    <t>0000138798</t>
+    <t>0000138675</t>
+  </si>
+  <si>
+    <t>BLF082</t>
+  </si>
+  <si>
+    <t>0000138676</t>
+  </si>
+  <si>
+    <t>BLF020</t>
+  </si>
+  <si>
+    <t>0000138866</t>
   </si>
   <si>
     <t>BLE055</t>
   </si>
   <si>
-    <t>0000138809</t>
+    <t>0000138869</t>
+  </si>
+  <si>
+    <t>BLE026</t>
+  </si>
+  <si>
+    <t>0000138892</t>
   </si>
   <si>
     <t>BLF046</t>
   </si>
   <si>
-    <t>0000138813</t>
+    <t>0000138871</t>
   </si>
   <si>
     <t>BLD087</t>
   </si>
   <si>
-    <t>0000138814</t>
-  </si>
-  <si>
-    <t>FR.01.05.01.03</t>
-  </si>
-  <si>
-    <t>0000138316</t>
-  </si>
-  <si>
-    <t>0000138755</t>
-  </si>
-  <si>
-    <t>FUMO</t>
-  </si>
-  <si>
-    <t>BLD062</t>
-  </si>
-  <si>
-    <t>0000138812</t>
+    <t>0000138872</t>
+  </si>
+  <si>
+    <t>BLE010</t>
+  </si>
+  <si>
+    <t>0000138906</t>
+  </si>
+  <si>
+    <t>BLD030</t>
+  </si>
+  <si>
+    <t>0000138922</t>
+  </si>
+  <si>
+    <t>BLE049</t>
+  </si>
+  <si>
+    <t>0000138932</t>
+  </si>
+  <si>
+    <t>BLE018</t>
+  </si>
+  <si>
+    <t>0000138921</t>
+  </si>
+  <si>
+    <t>BLD088</t>
+  </si>
+  <si>
+    <t>0000138926</t>
+  </si>
+  <si>
+    <t>BLD050</t>
+  </si>
+  <si>
+    <t>0000138900</t>
+  </si>
+  <si>
+    <t>BLF013</t>
+  </si>
+  <si>
+    <t>0000138896</t>
+  </si>
+  <si>
+    <t>FR.01.01.01.01</t>
+  </si>
+  <si>
+    <t>0000138756</t>
+  </si>
+  <si>
+    <t>BLD039</t>
+  </si>
+  <si>
+    <t>0000138895</t>
+  </si>
+  <si>
+    <t>BLD036</t>
+  </si>
+  <si>
+    <t>0000138904</t>
+  </si>
+  <si>
+    <t>BLD080</t>
+  </si>
+  <si>
+    <t>0000138927</t>
+  </si>
+  <si>
+    <t>BLF044</t>
+  </si>
+  <si>
+    <t>0000138894</t>
+  </si>
+  <si>
+    <t>BLE013</t>
+  </si>
+  <si>
+    <t>0000138925</t>
+  </si>
+  <si>
+    <t>BLE067</t>
+  </si>
+  <si>
+    <t>0000138924</t>
+  </si>
+  <si>
+    <t>BLG005</t>
+  </si>
+  <si>
+    <t>0000138923</t>
+  </si>
+  <si>
+    <t>BOX P</t>
+  </si>
+  <si>
+    <t>BLD065</t>
+  </si>
+  <si>
+    <t>0000138903</t>
   </si>
   <si>
     <t>NINE</t>
@@ -106,40 +211,145 @@
     <t>BLG072</t>
   </si>
   <si>
-    <t>0000138836</t>
+    <t>0000138913</t>
+  </si>
+  <si>
+    <t>0000138914</t>
+  </si>
+  <si>
+    <t>BLH080</t>
+  </si>
+  <si>
+    <t>0000138912</t>
+  </si>
+  <si>
+    <t>BLD044</t>
+  </si>
+  <si>
+    <t>0000138918</t>
+  </si>
+  <si>
+    <t>BLF059</t>
+  </si>
+  <si>
+    <t>0000138919</t>
   </si>
   <si>
     <t>BLD058</t>
   </si>
   <si>
-    <t>0000138837</t>
+    <t>0000138920</t>
   </si>
   <si>
     <t>SLIVE</t>
   </si>
   <si>
-    <t>BLD001</t>
-  </si>
-  <si>
-    <t>0000138810</t>
-  </si>
-  <si>
     <t>BLD073</t>
   </si>
   <si>
-    <t>0000138811</t>
-  </si>
-  <si>
-    <t>BLF078</t>
-  </si>
-  <si>
-    <t>0000138825</t>
+    <t>0000138870</t>
+  </si>
+  <si>
+    <t>BLC054</t>
+  </si>
+  <si>
+    <t>0000138908</t>
+  </si>
+  <si>
+    <t>BLC046</t>
+  </si>
+  <si>
+    <t>0000138898</t>
+  </si>
+  <si>
+    <t>BLE056</t>
+  </si>
+  <si>
+    <t>0000138897</t>
+  </si>
+  <si>
+    <t>BLH011</t>
+  </si>
+  <si>
+    <t>0000138899</t>
+  </si>
+  <si>
+    <t>BLC018</t>
+  </si>
+  <si>
+    <t>0000138880</t>
+  </si>
+  <si>
+    <t>BLD059</t>
+  </si>
+  <si>
+    <t>0000138881</t>
+  </si>
+  <si>
+    <t>BLE027</t>
+  </si>
+  <si>
+    <t>0000138882</t>
+  </si>
+  <si>
+    <t>BLF062</t>
+  </si>
+  <si>
+    <t>0000138879</t>
+  </si>
+  <si>
+    <t>BLG029</t>
+  </si>
+  <si>
+    <t>0000138883</t>
+  </si>
+  <si>
+    <t>BLE017</t>
+  </si>
+  <si>
+    <t>0000138890</t>
+  </si>
+  <si>
+    <t>BLE053</t>
+  </si>
+  <si>
+    <t>0000138889</t>
+  </si>
+  <si>
+    <t>BLF010</t>
+  </si>
+  <si>
+    <t>0000138891</t>
+  </si>
+  <si>
+    <t>BLG046</t>
+  </si>
+  <si>
+    <t>0000138888</t>
+  </si>
+  <si>
+    <t>BLD055</t>
+  </si>
+  <si>
+    <t>0000138902</t>
+  </si>
+  <si>
+    <t>BLE039</t>
+  </si>
+  <si>
+    <t>0000138901</t>
   </si>
   <si>
     <t>BLD007</t>
   </si>
   <si>
-    <t>0000138826</t>
+    <t>0000138884</t>
+  </si>
+  <si>
+    <t>BLD053</t>
+  </si>
+  <si>
+    <t>0000138885</t>
   </si>
   <si>
     <t>SLIVE P</t>
@@ -148,13 +358,13 @@
     <t>BLH079</t>
   </si>
   <si>
-    <t>0000138807</t>
+    <t>0000138867</t>
   </si>
   <si>
     <t>BLE030</t>
   </si>
   <si>
-    <t>0000138808</t>
+    <t>0000138868</t>
   </si>
 </sst>
 </file>
@@ -847,6 +1057,1371 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Picture 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Picture 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Picture 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="34" name="Picture 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Picture 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Picture 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="37" name="Picture 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="Picture 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="Picture 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="Picture 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Picture 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="43" name="Picture 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="44" name="Picture 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="45" name="Picture 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="46" name="Picture 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="47" name="Picture 47">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="48" name="Picture 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="49" name="Picture 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId50" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>77999</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>87999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1666875" cy="333375"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Picture 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId51" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1188,7 +2763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -1240,107 +2815,107 @@
         <v>11</v>
       </c>
       <c r="B4" s="3">
-        <v>10231474</v>
+        <v>10208005</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="3">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3">
-        <v>10215641</v>
+        <v>10208005</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="3">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>10224293</v>
+        <v>10215641</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3">
-        <v>10226339</v>
+        <v>10215641</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="3">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
-        <v>10226359</v>
+        <v>10223435</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3">
-        <v>10226363</v>
+        <v>10224293</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>23</v>
@@ -1352,207 +2927,907 @@
         <v>24</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3">
-        <v>10226363</v>
+        <v>10225180</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="B11" s="3">
-        <v>10230675</v>
+        <v>10226339</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D11" s="3">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
+        <v>10226359</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="3">
-        <v>10226368</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3">
+        <v>20</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="3">
-        <v>40</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="F12" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>10238738</v>
+        <v>10226380</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="3">
+        <v>80</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="3">
-        <v>40</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="F13" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3">
+        <v>10226386</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="3">
+        <v>40</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="3">
-        <v>10198819</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="3">
-        <v>70</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="F14" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3">
-        <v>10198819</v>
+        <v>10226386</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3">
-        <v>10226417</v>
+        <v>10226388</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D16" s="3">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="B17" s="3">
-        <v>10231475</v>
+        <v>10226404</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D17" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="B18" s="3">
-        <v>10223108</v>
+        <v>10226415</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D18" s="3">
         <v>20</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="3">
+        <v>10226425</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="3">
+      <c r="D19" s="3">
+        <v>90</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="3">
+        <v>10226425</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="3">
+        <v>10</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="3">
+        <v>10226428</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="3">
+        <v>10</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="3">
+        <v>10226435</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3">
+        <v>20</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" s="3">
+        <v>10226442</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="3">
+        <v>10</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="3">
+        <v>10226454</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="3">
+        <v>80</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="3">
+        <v>10242293</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="3">
+        <v>110</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="3">
+        <v>10242293</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="3">
+        <v>30</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="3">
+        <v>10242293</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="3">
+        <v>40</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="3">
+        <v>10226410</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="3">
+        <v>10</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="3">
+        <v>10226368</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="3">
+        <v>20</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="3">
+        <v>10226368</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="3">
+        <v>140</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="3">
+        <v>10238702</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="3">
+        <v>90</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="3">
+        <v>10238737</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" s="3">
+        <v>40</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="3">
+        <v>10238737</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="3">
+        <v>80</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="3">
+        <v>10238738</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" s="3">
+        <v>20</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="3">
+        <v>10198819</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" s="3">
+        <v>60</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B36" s="3">
+        <v>10208167</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="3">
+        <v>40</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B37" s="3">
+        <v>10226397</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D37" s="3">
+        <v>10</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" s="3">
+        <v>10226402</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="3">
+        <v>20</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" s="3">
+        <v>10226403</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D39" s="3">
+        <v>40</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D40" s="3">
+        <v>10</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D41" s="3">
+        <v>10</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D42" s="3">
+        <v>10</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D43" s="3">
+        <v>80</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="3">
+        <v>10226417</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D44" s="3">
+        <v>90</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="3">
+        <v>10226429</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D45" s="3">
+        <v>20</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B46" s="3">
+        <v>10226429</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D46" s="3">
+        <v>10</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B47" s="3">
+        <v>10226429</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D47" s="3">
+        <v>30</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B48" s="3">
+        <v>10226429</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D48" s="3">
+        <v>140</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49" s="3">
+        <v>10226452</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49" s="3">
+        <v>170</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50" s="3">
+        <v>10226452</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D50" s="3">
+        <v>30</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="3">
+        <v>10231475</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D51" s="3">
+        <v>10</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B52" s="3">
+        <v>10231484</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" s="3">
+        <v>10</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B53" s="3">
+        <v>10223108</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D53" s="3">
+        <v>40</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B54" s="3">
         <v>10226385</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="3">
+      <c r="C54" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D54" s="3">
         <v>10</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>11</v>
+      <c r="E54" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>